<commit_message>
Thème 2 — LOT 09 : Le jardin connecté (îlot 4e_C4 complet, 9 codes) — nouvel objet-fil de 4e
</commit_message>
<xml_diff>
--- a/_progressions/4e/Progression_Techno_4e_2026-2027_Martinique.xlsx
+++ b/_progressions/4e/Progression_Techno_4e_2026-2027_Martinique.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="🏠 Accueil" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="📅 Calendrier" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="🗓 Frise de l'année" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="📚 Référentiel Cycle 4" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="📗 Référentiel 4e" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="🧭 Progression" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="S1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="S2" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="S3" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="S4" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="S5" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="S6" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="S7" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="⚙ Moteur" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🏠 Accueil" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 Calendrier" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🗓 Frise de l'année" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📚 Référentiel Cycle 4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📗 Référentiel 4e" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🧭 Progression" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚙ Moteur" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="B14" s="196" t="inlineStr">
         <is>
-          <t>✅ Partiel : QCM « Jardin connecté », « Automatisation », « eCall » (existants) · 🔜 séquence îlot 4e_C4 (Fable)</t>
+          <t>✅ « Le jardin connecté » (îlot 4e_C4 complet, LOT 09 : séquence 4 séances + QCM 30 q + synthèses) — séquence : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C4-decrire-et-caracteriser-lorganisation/4e/4e_C4.1/sequence_4e_C4.1-C4.9_jardin_connecte.html · QCM existants (Automatisation, eCall) en complément</t>
         </is>
       </c>
       <c r="C14" s="132" t="n"/>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="B14" s="196" t="inlineStr">
         <is>
-          <t>✅ Partiel : QCM réseaux existant (40 q IP/NFC/RFID/Zigbee) · 🔜 séquence (Fable)</t>
+          <t>✅ « Le jardin connecté » séance 3 (réseau, IP fixe, 3 pannes simulées — LOT 09) : https://pll-process.github.io/en-ligne-pour-le-cycle-4/theme-2-structure-fonctionnement-comportement/C4-decrire-et-caracteriser-lorganisation/4e/4e_C4.1/sequence_4e_C4.1-C4.9_jardin_connecte.html · QCM XXL réseaux existant en entraînement intensif</t>
         </is>
       </c>
       <c r="C14" s="132" t="n"/>

</xml_diff>